<commit_message>
Fix tennis slate grades: use lowercase direction and player keys.
Tennis graded workbooks expose direction/player columns in lowercase and omit Dir/Direction. Matrix aggregation, prop breakdowns, O/U splits, and player leaderboards skipped every row. Added row_bet_direction() and wired it through build_pick_tier_direction_agg, def subgrid filters, prop labels, and O/U stats. Extended player_table to read player/team from lowercase keys. Regenerated 2026-05-09 slate eval, JSON bundle, analysis tabs, and mobile/www copies.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-09.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-09.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E2" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F2" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G2" t="n">
-        <v>44.2</v>
+        <v>49.2</v>
       </c>
     </row>
     <row r="3">
@@ -500,13 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="G3" t="n">
+        <v>75.90000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -552,16 +555,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E5" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F5" t="n">
         <v>15</v>
       </c>
       <c r="G5" t="n">
-        <v>54.5</v>
+        <v>57.1</v>
       </c>
     </row>
     <row r="6">
@@ -636,16 +639,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>257</v>
+        <v>4032</v>
       </c>
       <c r="E8" t="n">
-        <v>126</v>
+        <v>676</v>
       </c>
       <c r="F8" t="n">
-        <v>131</v>
+        <v>3356</v>
       </c>
       <c r="G8" t="n">
-        <v>49</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="9">
@@ -665,16 +668,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>93</v>
+        <v>123</v>
       </c>
       <c r="E9" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="F9" t="n">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="G9" t="n">
-        <v>60.2</v>
+        <v>56.9</v>
       </c>
     </row>
     <row r="10">
@@ -1145,10 +1148,10 @@
         <v>65</v>
       </c>
       <c r="R2" t="n">
-        <v>48</v>
+        <v>53.1</v>
       </c>
       <c r="S2" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -1157,13 +1160,16 @@
         <v>0</v>
       </c>
       <c r="X2" t="n">
-        <v>48.3</v>
+        <v>26.8</v>
       </c>
       <c r="Y2" t="n">
-        <v>120</v>
+        <v>553</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0</v>
       </c>
       <c r="AA2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AB2" t="n">
         <v>48</v>
@@ -1178,10 +1184,10 @@
         <v>5</v>
       </c>
       <c r="AF2" t="n">
-        <v>64.5</v>
+        <v>56.2</v>
       </c>
       <c r="AG2" t="n">
-        <v>31</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3">
@@ -1214,8 +1220,11 @@
       <c r="Q3" t="n">
         <v>0</v>
       </c>
+      <c r="R3" t="n">
+        <v>100</v>
+      </c>
       <c r="S3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U3" t="n">
         <v>0</v>
@@ -1223,11 +1232,17 @@
       <c r="W3" t="n">
         <v>0</v>
       </c>
+      <c r="X3" t="n">
+        <v>14.4</v>
+      </c>
       <c r="Y3" t="n">
-        <v>0</v>
+        <v>388</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>75</v>
       </c>
       <c r="AA3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AC3" t="n">
         <v>0</v>
@@ -1235,8 +1250,11 @@
       <c r="AE3" t="n">
         <v>0</v>
       </c>
+      <c r="AF3" t="n">
+        <v>50</v>
+      </c>
       <c r="AG3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -1306,19 +1324,19 @@
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>54.3</v>
+        <v>21.1</v>
       </c>
       <c r="Y4" t="n">
-        <v>94</v>
+        <v>615</v>
       </c>
       <c r="AA4" t="n">
         <v>0</v>
       </c>
       <c r="AB4" t="n">
-        <v>80</v>
+        <v>83.3</v>
       </c>
       <c r="AC4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AD4" t="n">
         <v>50</v>
@@ -1372,11 +1390,17 @@
       <c r="W5" t="n">
         <v>0</v>
       </c>
+      <c r="X5" t="n">
+        <v>14.3</v>
+      </c>
       <c r="Y5" t="n">
-        <v>0</v>
+        <v>671</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>80</v>
       </c>
       <c r="AA5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AC5" t="n">
         <v>0</v>
@@ -1384,8 +1408,11 @@
       <c r="AE5" t="n">
         <v>0</v>
       </c>
+      <c r="AF5" t="n">
+        <v>66.7</v>
+      </c>
       <c r="AG5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -1427,11 +1454,17 @@
       <c r="W6" t="n">
         <v>0</v>
       </c>
+      <c r="X6" t="n">
+        <v>12.5</v>
+      </c>
       <c r="Y6" t="n">
-        <v>0</v>
+        <v>160</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>100</v>
       </c>
       <c r="AA6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC6" t="n">
         <v>0</v>
@@ -1498,10 +1531,10 @@
         <v>2073</v>
       </c>
       <c r="R7" t="n">
-        <v>44.2</v>
+        <v>49.2</v>
       </c>
       <c r="S7" t="n">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="U7" t="n">
         <v>0</v>
@@ -1510,19 +1543,22 @@
         <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>49</v>
+        <v>16.8</v>
       </c>
       <c r="Y7" t="n">
-        <v>257</v>
+        <v>4032</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>75.90000000000001</v>
       </c>
       <c r="AA7" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="AB7" t="n">
-        <v>54.5</v>
+        <v>57.1</v>
       </c>
       <c r="AC7" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="AD7" t="n">
         <v>58.3</v>
@@ -1531,10 +1567,10 @@
         <v>36</v>
       </c>
       <c r="AF7" t="n">
-        <v>60.2</v>
+        <v>56.9</v>
       </c>
       <c r="AG7" t="n">
-        <v>93</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync combined slate 2026-05-10 UI bundle and sport pipeline outputs.
Refresh ui_runner and mobile/www tickets/slate JSON and HTML after combined_slate_tickets rebuild; update void validator and ticket diversity reports, payout sample log, and latest MLB/NBA/NHL ranked artifacts.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-09.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-09.xlsx
@@ -610,16 +610,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F7" t="n">
         <v>15</v>
       </c>
       <c r="G7" t="n">
-        <v>58.3</v>
+        <v>59.5</v>
       </c>
     </row>
     <row r="8">
@@ -639,16 +639,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4032</v>
+        <v>4037</v>
       </c>
       <c r="E8" t="n">
         <v>676</v>
       </c>
       <c r="F8" t="n">
-        <v>3356</v>
+        <v>3361</v>
       </c>
       <c r="G8" t="n">
-        <v>16.8</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="9">
@@ -668,16 +668,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E9" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F9" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G9" t="n">
-        <v>56.9</v>
+        <v>56.3</v>
       </c>
     </row>
     <row r="10">
@@ -697,16 +697,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>561</v>
+        <v>594</v>
       </c>
       <c r="E10" t="n">
-        <v>383</v>
+        <v>396</v>
       </c>
       <c r="F10" t="n">
-        <v>178</v>
+        <v>198</v>
       </c>
       <c r="G10" t="n">
-        <v>68.3</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="11">
@@ -726,16 +726,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>355</v>
+        <v>378</v>
       </c>
       <c r="E11" t="n">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="F11" t="n">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="G11" t="n">
-        <v>67.59999999999999</v>
+        <v>65.90000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -755,16 +755,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="E12" t="n">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="F12" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G12" t="n">
-        <v>65.09999999999999</v>
+        <v>65.40000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -813,16 +813,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="E14" t="n">
         <v>16</v>
       </c>
       <c r="F14" t="n">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="G14" t="n">
-        <v>22.5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15">
@@ -842,16 +842,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E15" t="n">
         <v>12</v>
       </c>
       <c r="F15" t="n">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="G15" t="n">
-        <v>16.4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16">
@@ -900,16 +900,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2073</v>
+        <v>2295</v>
       </c>
       <c r="E17" t="n">
-        <v>416</v>
+        <v>428</v>
       </c>
       <c r="F17" t="n">
-        <v>1657</v>
+        <v>1867</v>
       </c>
       <c r="G17" t="n">
-        <v>20.1</v>
+        <v>18.6</v>
       </c>
     </row>
   </sheetData>
@@ -1483,22 +1483,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>68.3</v>
+        <v>66.7</v>
       </c>
       <c r="C7" t="n">
-        <v>561</v>
+        <v>594</v>
       </c>
       <c r="D7" t="n">
-        <v>67.59999999999999</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>355</v>
+        <v>378</v>
       </c>
       <c r="F7" t="n">
-        <v>65.09999999999999</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="H7" t="n">
         <v>55.8</v>
@@ -1507,16 +1507,16 @@
         <v>154</v>
       </c>
       <c r="J7" t="n">
-        <v>22.5</v>
+        <v>20</v>
       </c>
       <c r="K7" t="n">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="L7" t="n">
-        <v>16.4</v>
+        <v>15</v>
       </c>
       <c r="M7" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="N7" t="n">
         <v>27.5</v>
@@ -1525,10 +1525,10 @@
         <v>40</v>
       </c>
       <c r="P7" t="n">
-        <v>20.1</v>
+        <v>18.6</v>
       </c>
       <c r="Q7" t="n">
-        <v>2073</v>
+        <v>2295</v>
       </c>
       <c r="R7" t="n">
         <v>49.2</v>
@@ -1543,10 +1543,10 @@
         <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>16.8</v>
+        <v>16.7</v>
       </c>
       <c r="Y7" t="n">
-        <v>4032</v>
+        <v>4037</v>
       </c>
       <c r="Z7" t="n">
         <v>75.90000000000001</v>
@@ -1561,16 +1561,16 @@
         <v>35</v>
       </c>
       <c r="AD7" t="n">
-        <v>58.3</v>
+        <v>59.5</v>
       </c>
       <c r="AE7" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="AF7" t="n">
-        <v>56.9</v>
+        <v>56.3</v>
       </c>
       <c r="AG7" t="n">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh WNBA L5 slate and combined UI for 2026-05-10.
Re-run WNBA pipeline with default 2025 stat window and combined slate; update ESPN cache, slate_latest and sport JSON, tickets, and related reports.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-09.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-09.xlsx
@@ -697,16 +697,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>594</v>
+        <v>602</v>
       </c>
       <c r="E10" t="n">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="F10" t="n">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="G10" t="n">
-        <v>66.7</v>
+        <v>66.8</v>
       </c>
     </row>
     <row r="11">
@@ -729,13 +729,13 @@
         <v>378</v>
       </c>
       <c r="E11" t="n">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="F11" t="n">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="G11" t="n">
-        <v>65.90000000000001</v>
+        <v>67.5</v>
       </c>
     </row>
     <row r="12">
@@ -758,13 +758,13 @@
         <v>156</v>
       </c>
       <c r="E12" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F12" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G12" t="n">
-        <v>65.40000000000001</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13">
@@ -900,16 +900,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2295</v>
+        <v>2319</v>
       </c>
       <c r="E17" t="n">
-        <v>428</v>
+        <v>437</v>
       </c>
       <c r="F17" t="n">
-        <v>1867</v>
+        <v>1882</v>
       </c>
       <c r="G17" t="n">
-        <v>18.6</v>
+        <v>18.8</v>
       </c>
     </row>
   </sheetData>
@@ -1483,19 +1483,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>66.7</v>
+        <v>66.8</v>
       </c>
       <c r="C7" t="n">
-        <v>594</v>
+        <v>602</v>
       </c>
       <c r="D7" t="n">
-        <v>65.90000000000001</v>
+        <v>67.5</v>
       </c>
       <c r="E7" t="n">
         <v>378</v>
       </c>
       <c r="F7" t="n">
-        <v>65.40000000000001</v>
+        <v>66</v>
       </c>
       <c r="G7" t="n">
         <v>156</v>
@@ -1525,10 +1525,10 @@
         <v>40</v>
       </c>
       <c r="P7" t="n">
-        <v>18.6</v>
+        <v>18.8</v>
       </c>
       <c r="Q7" t="n">
-        <v>2295</v>
+        <v>2319</v>
       </c>
       <c r="R7" t="n">
         <v>49.2</v>

</xml_diff>

<commit_message>
Daily slate 2026-05-11 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-09.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-09.xlsx
@@ -610,16 +610,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F7" t="n">
         <v>15</v>
       </c>
       <c r="G7" t="n">
-        <v>59.5</v>
+        <v>60.5</v>
       </c>
     </row>
     <row r="8">
@@ -639,13 +639,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4037</v>
+        <v>4044</v>
       </c>
       <c r="E8" t="n">
         <v>676</v>
       </c>
       <c r="F8" t="n">
-        <v>3361</v>
+        <v>3368</v>
       </c>
       <c r="G8" t="n">
         <v>16.7</v>
@@ -668,16 +668,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E9" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F9" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G9" t="n">
-        <v>56.3</v>
+        <v>56.2</v>
       </c>
     </row>
     <row r="10">
@@ -697,16 +697,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>602</v>
+        <v>613</v>
       </c>
       <c r="E10" t="n">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="F10" t="n">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="G10" t="n">
-        <v>66.8</v>
+        <v>66.09999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -726,16 +726,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>378</v>
+        <v>387</v>
       </c>
       <c r="E11" t="n">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="F11" t="n">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="G11" t="n">
-        <v>67.5</v>
+        <v>67.40000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -755,16 +755,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E12" t="n">
         <v>103</v>
       </c>
       <c r="F12" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G12" t="n">
-        <v>66</v>
+        <v>65.2</v>
       </c>
     </row>
     <row r="13">
@@ -813,16 +813,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E14" t="n">
         <v>16</v>
       </c>
       <c r="F14" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G14" t="n">
-        <v>20</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="15">
@@ -842,16 +842,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="E15" t="n">
         <v>12</v>
       </c>
       <c r="F15" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G15" t="n">
-        <v>15</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="16">
@@ -900,16 +900,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2319</v>
+        <v>2416</v>
       </c>
       <c r="E17" t="n">
-        <v>437</v>
+        <v>450</v>
       </c>
       <c r="F17" t="n">
-        <v>1882</v>
+        <v>1966</v>
       </c>
       <c r="G17" t="n">
-        <v>18.8</v>
+        <v>18.6</v>
       </c>
     </row>
   </sheetData>
@@ -1391,10 +1391,10 @@
         <v>0</v>
       </c>
       <c r="X5" t="n">
-        <v>14.3</v>
+        <v>14.2</v>
       </c>
       <c r="Y5" t="n">
-        <v>671</v>
+        <v>676</v>
       </c>
       <c r="Z5" t="n">
         <v>80</v>
@@ -1483,22 +1483,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>66.8</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="C7" t="n">
-        <v>602</v>
+        <v>613</v>
       </c>
       <c r="D7" t="n">
-        <v>67.5</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>378</v>
+        <v>387</v>
       </c>
       <c r="F7" t="n">
-        <v>66</v>
+        <v>65.2</v>
       </c>
       <c r="G7" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H7" t="n">
         <v>55.8</v>
@@ -1507,16 +1507,16 @@
         <v>154</v>
       </c>
       <c r="J7" t="n">
-        <v>20</v>
+        <v>19.5</v>
       </c>
       <c r="K7" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="L7" t="n">
-        <v>15</v>
+        <v>14.5</v>
       </c>
       <c r="M7" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="N7" t="n">
         <v>27.5</v>
@@ -1525,10 +1525,10 @@
         <v>40</v>
       </c>
       <c r="P7" t="n">
-        <v>18.8</v>
+        <v>18.6</v>
       </c>
       <c r="Q7" t="n">
-        <v>2319</v>
+        <v>2416</v>
       </c>
       <c r="R7" t="n">
         <v>49.2</v>
@@ -1546,7 +1546,7 @@
         <v>16.7</v>
       </c>
       <c r="Y7" t="n">
-        <v>4037</v>
+        <v>4044</v>
       </c>
       <c r="Z7" t="n">
         <v>75.90000000000001</v>
@@ -1561,16 +1561,16 @@
         <v>35</v>
       </c>
       <c r="AD7" t="n">
-        <v>59.5</v>
+        <v>60.5</v>
       </c>
       <c r="AE7" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="AF7" t="n">
-        <v>56.3</v>
+        <v>56.2</v>
       </c>
       <c r="AG7" t="n">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>